<commit_message>
add new field Raw Material Type
</commit_message>
<xml_diff>
--- a/template/Raw_Mat_Template.xlsx
+++ b/template/Raw_Mat_Template.xlsx
@@ -1,33 +1,50 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>工作表</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>Sheet1</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Yeong Kin Rong</dc:creator>
+  <cp:lastModifiedBy>Jih Bin Ng</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2025-03-02T12:51:00Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-06-01T07:18:45Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="ICV">
+    <vt:lpwstr>EA19161D75D24265A1A26E906A87F1DE_12</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="KSOProductBuildVer">
+    <vt:lpwstr>1033-12.1.0.25180</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="CalculationRule">
+    <vt:i4>0</vt:i4>
+  </property>
+</Properties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Code</t>
   </si>
@@ -35,12 +52,15 @@
     <t>Name</t>
   </si>
   <si>
+    <t>RawMaterialType</t>
+  </si>
+  <si>
     <t>Description</t>
   </si>
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -728,7 +748,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1003,13 +1023,40 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="27945" windowHeight="12180"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" outlineLevelCol="2"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="15.75" spans="1:3">
+    <row r="1" s="1" customFormat="1" ht="15.75" spans="1:4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1019,6 +1066,9 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update raw mat template and add checking for allowed raw mat type
</commit_message>
<xml_diff>
--- a/template/Raw_Mat_Template.xlsx
+++ b/template/Raw_Mat_Template.xlsx
@@ -1,49 +1,32 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel</Application>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>工作表</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>1</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="1" baseType="lpstr">
-      <vt:lpstr>Sheet1</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="27945" windowHeight="12180"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <dc:creator>Yeong Kin Rong</dc:creator>
-  <cp:lastModifiedBy>Jih Bin Ng</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2025-03-02T12:51:00Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-06-01T07:18:45Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="ICV">
-    <vt:lpwstr>EA19161D75D24265A1A26E906A87F1DE_12</vt:lpwstr>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="KSOProductBuildVer">
-    <vt:lpwstr>1033-12.1.0.25180</vt:lpwstr>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="CalculationRule">
-    <vt:i4>0</vt:i4>
-  </property>
-</Properties>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Code</t>
@@ -52,7 +35,7 @@
     <t>Name</t>
   </si>
   <si>
-    <t>RawMaterialType</t>
+    <t>Raw Material Type</t>
   </si>
   <si>
     <t>Description</t>
@@ -60,7 +43,7 @@
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -683,9 +666,8 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -748,7 +730,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1023,50 +1005,26 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" outlineLevelCol="3"/>
+  <cols>
+    <col min="3" max="3" width="16.4444444444444" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="15.75" spans="1:4">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>